<commit_message>
Données : Aircall S22 (202622), export tickets HubSpot 2026-06-01
Ajout des données support récentes et mises à jour associées (analyses,
scripts de traitement, docs de déploiement, config exemple).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Affid/analyse_appels_tickets/yelda_comex_analyse_utilisation.xlsx
+++ b/data/Affid/analyse_appels_tickets/yelda_comex_analyse_utilisation.xlsx
@@ -192,12 +192,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Volumetrie_hebdo'!$A$2:$A$18</f>
+              <f>'Volumetrie_hebdo'!$A$2:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Volumetrie_hebdo'!$C$2:$C$18</f>
+              <f>'Volumetrie_hebdo'!$C$2:$C$22</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Volumetrie_mensuelle'!$A$2:$A$5</f>
+              <f>'Volumetrie_mensuelle'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Volumetrie_mensuelle'!$B$2:$B$5</f>
+              <f>'Volumetrie_mensuelle'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -423,12 +423,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Satisfaction_LLM_mensuel'!$A$2:$A$5</f>
+              <f>'Satisfaction_LLM_mensuel'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Satisfaction_LLM_mensuel'!$F$2:$F$5</f>
+              <f>'Satisfaction_LLM_mensuel'!$F$2:$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -894,7 +894,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-01-01 → 2026-04-21</t>
+          <t>2026-01-01 → 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6446</v>
+        <v>7126</v>
       </c>
     </row>
     <row r="4">
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1317</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="5">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20.4</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="6">
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>888</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="7">
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>247</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="9">
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>221</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12">
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16.8</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="13">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1276</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="14">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>78.7</v>
+        <v>81.5</v>
       </c>
     </row>
   </sheetData>
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1468,16 +1468,112 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>12</v>
+        <v>89</v>
       </c>
       <c r="D18" t="n">
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="E18" t="n">
         <v>70</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-S18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>110</v>
+      </c>
+      <c r="D19" t="n">
+        <v>90</v>
+      </c>
+      <c r="E19" t="n">
+        <v>116</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-S19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>49</v>
+      </c>
+      <c r="D20" t="n">
+        <v>43</v>
+      </c>
+      <c r="E20" t="n">
+        <v>91</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-S20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>47</v>
+      </c>
+      <c r="D21" t="n">
+        <v>43</v>
+      </c>
+      <c r="E21" t="n">
+        <v>102</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-S21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>127</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1492,7 +1588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1593,15 +1689,34 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>166</v>
+        <v>336</v>
       </c>
       <c r="C5" t="n">
-        <v>134</v>
+        <v>253</v>
       </c>
       <c r="D5" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="E5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>116</v>
+      </c>
+      <c r="C6" t="n">
+        <v>97</v>
+      </c>
+      <c r="D6" t="n">
+        <v>92</v>
+      </c>
+      <c r="E6" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1643,7 +1758,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1317</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="3">
@@ -1653,7 +1768,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -1663,7 +1778,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>888</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="5">
@@ -1673,7 +1788,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>641</v>
+        <v>713</v>
       </c>
     </row>
     <row r="6">
@@ -1683,7 +1798,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>247</v>
+        <v>315</v>
       </c>
     </row>
     <row r="7">
@@ -1693,7 +1808,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>92</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8">
@@ -1703,7 +1818,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -1713,7 +1828,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.46</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="10">
@@ -1737,7 +1852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1853,19 +1968,41 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>142</v>
+        <v>301</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>148</v>
+        <v>318</v>
       </c>
       <c r="F5" t="n">
-        <v>95.90000000000001</v>
+        <v>94.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>109</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>116</v>
+      </c>
+      <c r="F6" t="n">
+        <v>94.8</v>
       </c>
     </row>
   </sheetData>
@@ -1880,7 +2017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1981,35 +2118,54 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>166</v>
+        <v>336</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="E5" t="n">
-        <v>96.40000000000001</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>116</v>
+      </c>
+      <c r="C6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>1317</v>
-      </c>
-      <c r="C6" t="n">
-        <v>221</v>
-      </c>
-      <c r="D6" t="n">
-        <v>16.8</v>
-      </c>
-      <c r="E6" t="n">
-        <v>83.2</v>
+      <c r="B7" t="n">
+        <v>1603</v>
+      </c>
+      <c r="C7" t="n">
+        <v>238</v>
+      </c>
+      <c r="D7" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>85.2</v>
       </c>
     </row>
   </sheetData>
@@ -2055,10 +2211,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>309</v>
+        <v>367</v>
       </c>
       <c r="C2" t="n">
-        <v>23.5</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="3">
@@ -2068,10 +2224,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>222</v>
+        <v>253</v>
       </c>
       <c r="C3" t="n">
-        <v>16.9</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="4">
@@ -2081,10 +2237,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>196</v>
+        <v>216</v>
       </c>
       <c r="C4" t="n">
-        <v>14.9</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="5">
@@ -2094,10 +2250,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="6">
@@ -2107,62 +2263,62 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="C6" t="n">
-        <v>8.4</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>contact_agent_phone</t>
+          <t>small_talk_thanks</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="C7" t="n">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>contact_agent_callback</t>
+          <t>small_talk_problem</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="C8" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>small_talk_thanks</t>
+          <t>contact_agent_phone</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="C9" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>small_talk_problem</t>
+          <t>contact_agent_callback</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="11">
@@ -2172,20 +2328,20 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C11" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>assistant_faq_help</t>
+          <t>small_talk_no</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C12" t="n">
         <v>2.7</v>
@@ -2194,27 +2350,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>small_talk_no</t>
+          <t>small_talk_not_good</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C13" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>small_talk_not_good</t>
+          <t>assistant_faq_help</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C14" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="15">
@@ -2224,7 +2380,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C15" t="n">
         <v>2.2</v>
@@ -2233,11 +2389,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>small_talk_not_happy</t>
+          <t>small_talk_incorrect</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C16" t="n">
         <v>2.1</v>
@@ -2246,24 +2402,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>small_talk_incorrect</t>
+          <t>request_job_openings</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C17" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>request_job_openings</t>
+          <t>small_talk_not_happy</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C18" t="n">
         <v>2</v>
@@ -2276,7 +2432,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C19" t="n">
         <v>1.7</v>
@@ -2285,27 +2441,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>assistant_run_cancel</t>
+          <t>assistant_run_main_menu</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C20" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>small_talk_yes</t>
+          <t>small_talk_insomnia</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C21" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>
@@ -2570,14 +2726,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Ouvertures du widget : 6446</t>
+          <t xml:space="preserve">  - Ouvertures du widget : 7126</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Conversations initiées : 1317 (20.4 %)</t>
+          <t xml:space="preserve">  - Conversations initiées : 1603 (22.5 %)</t>
         </is>
       </c>
     </row>

</xml_diff>